<commit_message>
K-Means App completa con tabla, centroides y métricas
</commit_message>
<xml_diff>
--- a/static/KMeans_Iteracion_1_Estudiantes (1).xlsx
+++ b/static/KMeans_Iteracion_1_Estudiantes (1).xlsx
@@ -1,15 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_284351E7EE6AFFF2C7C4BF3B74EE0FA1E88E0333" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\batle\machine-learning-exp\static\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB65B49-D638-4D79-A7F6-B260A585A42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Iteracion 1" sheetId="1" r:id="rId1"/>
-    <sheet name="Documentacion" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Iteracion 1'!$A$1:$G$101</definedName>
@@ -32,36 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
-  <si>
-    <t>Estudiante</t>
-  </si>
-  <si>
-    <t>Horas_Estudio</t>
-  </si>
-  <si>
-    <t>Calificacion</t>
-  </si>
-  <si>
-    <t>Distancia_C1</t>
-  </si>
-  <si>
-    <t>Distancia_C2</t>
-  </si>
-  <si>
-    <t>Distancia_C3</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>Cluster</t>
-  </si>
-  <si>
-    <t>Centroides iniciales</t>
-  </si>
-  <si>
-    <t>Centroide</t>
-  </si>
-  <si>
-    <t>Horas</t>
   </si>
   <si>
     <t>C1</t>
@@ -73,77 +50,47 @@
     <t>C3</t>
   </si>
   <si>
-    <t>Nuevos centroides - Iteración 1</t>
+    <t>Student</t>
   </si>
   <si>
-    <t>Nuevo X</t>
+    <t>Study_Hours</t>
   </si>
   <si>
-    <t>Nuevo Y</t>
+    <t>Calification</t>
   </si>
   <si>
-    <t>Tema</t>
+    <t>Distance_C1</t>
   </si>
   <si>
-    <t>Segmentación de estudiantes según horas de estudio y rendimiento académico.</t>
+    <t>Distance_C2</t>
   </si>
   <si>
-    <t>Variable X</t>
+    <t>Distance_C3</t>
   </si>
   <si>
-    <t>Horas de estudio por semana.</t>
+    <t>Initials Centroids</t>
   </si>
   <si>
-    <t>Variable Y</t>
+    <t>Centroid</t>
   </si>
   <si>
-    <t>Calificación promedio sobre 100.</t>
+    <t>Hours</t>
   </si>
   <si>
-    <t>Registros</t>
+    <t>New centroids - Iteration 1</t>
   </si>
   <si>
-    <t>100 estudiantes.</t>
+    <t>New X</t>
   </si>
   <si>
-    <t>Número de clusters</t>
-  </si>
-  <si>
-    <t>3.</t>
-  </si>
-  <si>
-    <t>C1=(3,45), C2=(8,65), C3=(14,85).</t>
-  </si>
-  <si>
-    <t>Distancia</t>
-  </si>
-  <si>
-    <t>d = √((X-Xc)² + (Y-Yc)²).</t>
-  </si>
-  <si>
-    <t>Asignación</t>
-  </si>
-  <si>
-    <t>Cada estudiante se asigna al centroide con menor distancia.</t>
-  </si>
-  <si>
-    <t>Actualización</t>
-  </si>
-  <si>
-    <t>Cada nuevo centroide se obtiene promediando X e Y de los estudiantes asignados.</t>
-  </si>
-  <si>
-    <t>Nota</t>
-  </si>
-  <si>
-    <t>Las fórmulas de la hoja 'Iteracion 1' realizan automáticamente los cálculos de la primera iteración.</t>
+    <t>New Y</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -154,11 +101,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -187,13 +129,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,37 +438,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G113"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.98828125" customWidth="1"/>
-    <col min="2" max="6" width="16.0078125" customWidth="1"/>
-    <col min="7" max="7" width="11.97265625" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -538,23 +479,23 @@
         <v>45</v>
       </c>
       <c r="D2">
-        <f>SQRT((B2-$B$105)^2+(C2-$C$105)^2)</f>
+        <f t="shared" ref="D2:D33" si="0">SQRT((B2-$B$105)^2+(C2-$C$105)^2)</f>
         <v>1</v>
       </c>
       <c r="E2">
-        <f>SQRT((B2-$B$106)^2+(C2-$C$106)^2)</f>
+        <f t="shared" ref="E2:E33" si="1">SQRT((B2-$B$106)^2+(C2-$C$106)^2)</f>
         <v>20.880613017821101</v>
       </c>
       <c r="F2">
-        <f>SQRT((B2-$B$107)^2+(C2-$C$107)^2)</f>
+        <f t="shared" ref="F2:F33" si="2">SQRT((B2-$B$107)^2+(C2-$C$107)^2)</f>
         <v>41.761226035642203</v>
       </c>
       <c r="G2" t="str">
-        <f>IF(D2=MIN(D2:F2),"C1",IF(E2=MIN(D2:F2),"C2","C3"))</f>
+        <f t="shared" ref="G2:G33" si="3">IF(D2=MIN(D2:F2),"C1",IF(E2=MIN(D2:F2),"C2","C3"))</f>
         <v>C1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -565,23 +506,23 @@
         <v>48</v>
       </c>
       <c r="D3">
-        <f>SQRT((B3-$B$105)^2+(C3-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="E3">
-        <f>SQRT((B3-$B$106)^2+(C3-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>17.720045146669349</v>
       </c>
       <c r="F3">
-        <f>SQRT((B3-$B$107)^2+(C3-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>38.600518131237564</v>
       </c>
       <c r="G3" t="str">
-        <f>IF(D3=MIN(D3:F3),"C1",IF(E3=MIN(D3:F3),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -592,23 +533,23 @@
         <v>50</v>
       </c>
       <c r="D4">
-        <f>SQRT((B4-$B$105)^2+(C4-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>5.0990195135927845</v>
       </c>
       <c r="E4">
-        <f>SQRT((B4-$B$106)^2+(C4-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>15.524174696260024</v>
       </c>
       <c r="F4">
-        <f>SQRT((B4-$B$107)^2+(C4-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>36.400549446402593</v>
       </c>
       <c r="G4" t="str">
-        <f>IF(D4=MIN(D4:F4),"C1",IF(E4=MIN(D4:F4),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -619,23 +560,23 @@
         <v>42</v>
       </c>
       <c r="D5">
-        <f>SQRT((B5-$B$105)^2+(C5-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>3.1622776601683795</v>
       </c>
       <c r="E5">
-        <f>SQRT((B5-$B$106)^2+(C5-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>23.769728648009426</v>
       </c>
       <c r="F5">
-        <f>SQRT((B5-$B$107)^2+(C5-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>44.643028571099428</v>
       </c>
       <c r="G5" t="str">
-        <f>IF(D5=MIN(D5:F5),"C1",IF(E5=MIN(D5:F5),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -646,23 +587,23 @@
         <v>53</v>
       </c>
       <c r="D6">
-        <f>SQRT((B6-$B$105)^2+(C6-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>8.2462112512353212</v>
       </c>
       <c r="E6">
-        <f>SQRT((B6-$B$106)^2+(C6-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>12.369316876852981</v>
       </c>
       <c r="F6">
-        <f>SQRT((B6-$B$107)^2+(C6-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>33.241540277189323</v>
       </c>
       <c r="G6" t="str">
-        <f>IF(D6=MIN(D6:F6),"C1",IF(E6=MIN(D6:F6),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -673,23 +614,23 @@
         <v>47</v>
       </c>
       <c r="D7">
-        <f>SQRT((B7-$B$105)^2+(C7-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>2.2360679774997898</v>
       </c>
       <c r="E7">
-        <f>SQRT((B7-$B$106)^2+(C7-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>18.439088914585774</v>
       </c>
       <c r="F7">
-        <f>SQRT((B7-$B$107)^2+(C7-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>39.293765408776999</v>
       </c>
       <c r="G7" t="str">
-        <f>IF(D7=MIN(D7:F7),"C1",IF(E7=MIN(D7:F7),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -700,23 +641,23 @@
         <v>44</v>
       </c>
       <c r="D8">
-        <f>SQRT((B8-$B$105)^2+(C8-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E8">
-        <f>SQRT((B8-$B$106)^2+(C8-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>21.587033144922902</v>
       </c>
       <c r="F8">
-        <f>SQRT((B8-$B$107)^2+(C8-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>42.449970553582247</v>
       </c>
       <c r="G8" t="str">
-        <f>IF(D8=MIN(D8:F8),"C1",IF(E8=MIN(D8:F8),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -727,23 +668,23 @@
         <v>55</v>
       </c>
       <c r="D9">
-        <f>SQRT((B9-$B$105)^2+(C9-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>10.198039027185569</v>
       </c>
       <c r="E9">
-        <f>SQRT((B9-$B$106)^2+(C9-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>10.440306508910551</v>
       </c>
       <c r="F9">
-        <f>SQRT((B9-$B$107)^2+(C9-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>31.32091952673165</v>
       </c>
       <c r="G9" t="str">
-        <f>IF(D9=MIN(D9:F9),"C1",IF(E9=MIN(D9:F9),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -754,23 +695,23 @@
         <v>58</v>
       </c>
       <c r="D10">
-        <f>SQRT((B10-$B$105)^2+(C10-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>13.341664064126334</v>
       </c>
       <c r="E10">
-        <f>SQRT((B10-$B$106)^2+(C10-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>7.2801098892805181</v>
       </c>
       <c r="F10">
-        <f>SQRT((B10-$B$107)^2+(C10-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>28.160255680657446</v>
       </c>
       <c r="G10" t="str">
-        <f>IF(D10=MIN(D10:F10),"C1",IF(E10=MIN(D10:F10),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -781,23 +722,23 @@
         <v>52</v>
       </c>
       <c r="D11">
-        <f>SQRT((B11-$B$105)^2+(C11-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>7.0710678118654755</v>
       </c>
       <c r="E11">
-        <f>SQRT((B11-$B$106)^2+(C11-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>13.601470508735444</v>
       </c>
       <c r="F11">
-        <f>SQRT((B11-$B$107)^2+(C11-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>34.481879299133332</v>
       </c>
       <c r="G11" t="str">
-        <f>IF(D11=MIN(D11:F11),"C1",IF(E11=MIN(D11:F11),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -808,23 +749,23 @@
         <v>46</v>
       </c>
       <c r="D12">
-        <f>SQRT((B12-$B$105)^2+(C12-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="E12">
-        <f>SQRT((B12-$B$106)^2+(C12-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>19.924858845171276</v>
       </c>
       <c r="F12">
-        <f>SQRT((B12-$B$107)^2+(C12-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>40.80441152620633</v>
       </c>
       <c r="G12" t="str">
-        <f>IF(D12=MIN(D12:F12),"C1",IF(E12=MIN(D12:F12),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -835,23 +776,23 @@
         <v>51</v>
       </c>
       <c r="D13">
-        <f>SQRT((B13-$B$105)^2+(C13-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="E13">
-        <f>SQRT((B13-$B$106)^2+(C13-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>14.866068747318506</v>
       </c>
       <c r="F13">
-        <f>SQRT((B13-$B$107)^2+(C13-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>35.735136770411273</v>
       </c>
       <c r="G13" t="str">
-        <f>IF(D13=MIN(D13:F13),"C1",IF(E13=MIN(D13:F13),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -862,23 +803,23 @@
         <v>49</v>
       </c>
       <c r="D14">
-        <f>SQRT((B14-$B$105)^2+(C14-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>4.4721359549995796</v>
       </c>
       <c r="E14">
-        <f>SQRT((B14-$B$106)^2+(C14-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>16.278820596099706</v>
       </c>
       <c r="F14">
-        <f>SQRT((B14-$B$107)^2+(C14-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>37.107950630558946</v>
       </c>
       <c r="G14" t="str">
-        <f>IF(D14=MIN(D14:F14),"C1",IF(E14=MIN(D14:F14),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -889,23 +830,23 @@
         <v>54</v>
       </c>
       <c r="D15">
-        <f>SQRT((B15-$B$105)^2+(C15-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>9.0553851381374173</v>
       </c>
       <c r="E15">
-        <f>SQRT((B15-$B$106)^2+(C15-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>11.704699910719626</v>
       </c>
       <c r="F15">
-        <f>SQRT((B15-$B$107)^2+(C15-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>32.572994949804659</v>
       </c>
       <c r="G15" t="str">
-        <f>IF(D15=MIN(D15:F15),"C1",IF(E15=MIN(D15:F15),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -916,23 +857,23 @@
         <v>56</v>
       </c>
       <c r="D16">
-        <f>SQRT((B16-$B$105)^2+(C16-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>11.401754250991379</v>
       </c>
       <c r="E16">
-        <f>SQRT((B16-$B$106)^2+(C16-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>9.2195444572928871</v>
       </c>
       <c r="F16">
-        <f>SQRT((B16-$B$107)^2+(C16-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>30.083217912982647</v>
       </c>
       <c r="G16" t="str">
-        <f>IF(D16=MIN(D16:F16),"C1",IF(E16=MIN(D16:F16),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -943,23 +884,23 @@
         <v>46</v>
       </c>
       <c r="D17">
-        <f>SQRT((B17-$B$105)^2+(C17-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E17">
-        <f>SQRT((B17-$B$106)^2+(C17-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>19.646882704388499</v>
       </c>
       <c r="F17">
-        <f>SQRT((B17-$B$107)^2+(C17-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>40.521599178709621</v>
       </c>
       <c r="G17" t="str">
-        <f>IF(D17=MIN(D17:F17),"C1",IF(E17=MIN(D17:F17),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -970,23 +911,23 @@
         <v>52</v>
       </c>
       <c r="D18">
-        <f>SQRT((B18-$B$105)^2+(C18-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>7.2801098892805181</v>
       </c>
       <c r="E18">
-        <f>SQRT((B18-$B$106)^2+(C18-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>13.341664064126334</v>
       </c>
       <c r="F18">
-        <f>SQRT((B18-$B$107)^2+(C18-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>34.205262752974143</v>
       </c>
       <c r="G18" t="str">
-        <f>IF(D18=MIN(D18:F18),"C1",IF(E18=MIN(D18:F18),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -997,23 +938,23 @@
         <v>43</v>
       </c>
       <c r="D19">
-        <f>SQRT((B19-$B$105)^2+(C19-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>2.2360679774997898</v>
       </c>
       <c r="E19">
-        <f>SQRT((B19-$B$106)^2+(C19-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>22.803508501982758</v>
       </c>
       <c r="F19">
-        <f>SQRT((B19-$B$107)^2+(C19-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>43.68065933568311</v>
       </c>
       <c r="G19" t="str">
-        <f>IF(D19=MIN(D19:F19),"C1",IF(E19=MIN(D19:F19),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1024,23 +965,23 @@
         <v>49</v>
       </c>
       <c r="D20">
-        <f>SQRT((B20-$B$105)^2+(C20-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>4.1231056256176606</v>
       </c>
       <c r="E20">
-        <f>SQRT((B20-$B$106)^2+(C20-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>16.492422502470642</v>
       </c>
       <c r="F20">
-        <f>SQRT((B20-$B$107)^2+(C20-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>37.363083384538811</v>
       </c>
       <c r="G20" t="str">
-        <f>IF(D20=MIN(D20:F20),"C1",IF(E20=MIN(D20:F20),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1051,23 +992,23 @@
         <v>60</v>
       </c>
       <c r="D21">
-        <f>SQRT((B21-$B$105)^2+(C21-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>15.297058540778355</v>
       </c>
       <c r="E21">
-        <f>SQRT((B21-$B$106)^2+(C21-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>5.3851648071345037</v>
       </c>
       <c r="F21">
-        <f>SQRT((B21-$B$107)^2+(C21-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>26.248809496813376</v>
       </c>
       <c r="G21" t="str">
-        <f>IF(D21=MIN(D21:F21),"C1",IF(E21=MIN(D21:F21),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1078,23 +1019,23 @@
         <v>62</v>
       </c>
       <c r="D22">
-        <f>SQRT((B22-$B$105)^2+(C22-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>17.464249196572979</v>
       </c>
       <c r="E22">
-        <f>SQRT((B22-$B$106)^2+(C22-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>3.1622776601683795</v>
       </c>
       <c r="F22">
-        <f>SQRT((B22-$B$107)^2+(C22-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>24.041630560342615</v>
       </c>
       <c r="G22" t="str">
-        <f>IF(D22=MIN(D22:F22),"C1",IF(E22=MIN(D22:F22),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1105,23 +1046,23 @@
         <v>65</v>
       </c>
       <c r="D23">
-        <f>SQRT((B23-$B$105)^2+(C23-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>20.615528128088304</v>
       </c>
       <c r="E23">
-        <f>SQRT((B23-$B$106)^2+(C23-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F23">
-        <f>SQRT((B23-$B$107)^2+(C23-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>20.880613017821101</v>
       </c>
       <c r="G23" t="str">
-        <f>IF(D23=MIN(D23:F23),"C1",IF(E23=MIN(D23:F23),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1132,23 +1073,23 @@
         <v>68</v>
       </c>
       <c r="D24">
-        <f>SQRT((B24-$B$105)^2+(C24-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>23.769728648009426</v>
       </c>
       <c r="E24">
-        <f>SQRT((B24-$B$106)^2+(C24-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>3.1622776601683795</v>
       </c>
       <c r="F24">
-        <f>SQRT((B24-$B$107)^2+(C24-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>17.720045146669349</v>
       </c>
       <c r="G24" t="str">
-        <f>IF(D24=MIN(D24:F24),"C1",IF(E24=MIN(D24:F24),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1159,23 +1100,23 @@
         <v>64</v>
       </c>
       <c r="D25">
-        <f>SQRT((B25-$B$105)^2+(C25-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>19.416487838947599</v>
       </c>
       <c r="E25">
-        <f>SQRT((B25-$B$106)^2+(C25-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="F25">
-        <f>SQRT((B25-$B$107)^2+(C25-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>22.135943621178654</v>
       </c>
       <c r="G25" t="str">
-        <f>IF(D25=MIN(D25:F25),"C1",IF(E25=MIN(D25:F25),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1186,23 +1127,23 @@
         <v>70</v>
       </c>
       <c r="D26">
-        <f>SQRT((B26-$B$105)^2+(C26-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>25.96150997149434</v>
       </c>
       <c r="E26">
-        <f>SQRT((B26-$B$106)^2+(C26-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>5.3851648071345037</v>
       </c>
       <c r="F26">
-        <f>SQRT((B26-$B$107)^2+(C26-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>15.524174696260024</v>
       </c>
       <c r="G26" t="str">
-        <f>IF(D26=MIN(D26:F26),"C1",IF(E26=MIN(D26:F26),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1213,23 +1154,23 @@
         <v>67</v>
       </c>
       <c r="D27">
-        <f>SQRT((B27-$B$105)^2+(C27-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>22.561028345356956</v>
       </c>
       <c r="E27">
-        <f>SQRT((B27-$B$106)^2+(C27-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="F27">
-        <f>SQRT((B27-$B$107)^2+(C27-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>18.973665961010276</v>
       </c>
       <c r="G27" t="str">
-        <f>IF(D27=MIN(D27:F27),"C1",IF(E27=MIN(D27:F27),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1240,23 +1181,23 @@
         <v>72</v>
       </c>
       <c r="D28">
-        <f>SQRT((B28-$B$105)^2+(C28-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>27.658633371878661</v>
       </c>
       <c r="E28">
-        <f>SQRT((B28-$B$106)^2+(C28-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>7.0710678118654755</v>
       </c>
       <c r="F28">
-        <f>SQRT((B28-$B$107)^2+(C28-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>13.928388277184119</v>
       </c>
       <c r="G28" t="str">
-        <f>IF(D28=MIN(D28:F28),"C1",IF(E28=MIN(D28:F28),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1267,23 +1208,23 @@
         <v>61</v>
       </c>
       <c r="D29">
-        <f>SQRT((B29-$B$105)^2+(C29-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>16.492422502470642</v>
       </c>
       <c r="E29">
-        <f>SQRT((B29-$B$106)^2+(C29-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>4.1231056256176606</v>
       </c>
       <c r="F29">
-        <f>SQRT((B29-$B$107)^2+(C29-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="G29" t="str">
-        <f>IF(D29=MIN(D29:F29),"C1",IF(E29=MIN(D29:F29),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1294,23 +1235,23 @@
         <v>74</v>
       </c>
       <c r="D30">
-        <f>SQRT((B30-$B$105)^2+(C30-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>29.832867780352597</v>
       </c>
       <c r="E30">
-        <f>SQRT((B30-$B$106)^2+(C30-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>9.2195444572928871</v>
       </c>
       <c r="F30">
-        <f>SQRT((B30-$B$107)^2+(C30-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>11.704699910719626</v>
       </c>
       <c r="G30" t="str">
-        <f>IF(D30=MIN(D30:F30),"C1",IF(E30=MIN(D30:F30),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1321,23 +1262,23 @@
         <v>69</v>
       </c>
       <c r="D31">
-        <f>SQRT((B31-$B$105)^2+(C31-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>24.515301344262525</v>
       </c>
       <c r="E31">
-        <f>SQRT((B31-$B$106)^2+(C31-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="F31">
-        <f>SQRT((B31-$B$107)^2+(C31-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>17.088007490635061</v>
       </c>
       <c r="G31" t="str">
-        <f>IF(D31=MIN(D31:F31),"C1",IF(E31=MIN(D31:F31),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1348,23 +1289,23 @@
         <v>71</v>
       </c>
       <c r="D32">
-        <f>SQRT((B32-$B$105)^2+(C32-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>26.683328128252668</v>
       </c>
       <c r="E32">
-        <f>SQRT((B32-$B$106)^2+(C32-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>6.0827625302982193</v>
       </c>
       <c r="F32">
-        <f>SQRT((B32-$B$107)^2+(C32-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>14.866068747318506</v>
       </c>
       <c r="G32" t="str">
-        <f>IF(D32=MIN(D32:F32),"C1",IF(E32=MIN(D32:F32),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1375,23 +1316,23 @@
         <v>66</v>
       </c>
       <c r="D33">
-        <f>SQRT((B33-$B$105)^2+(C33-$C$105)^2)</f>
+        <f t="shared" si="0"/>
         <v>21.377558326431949</v>
       </c>
       <c r="E33">
-        <f>SQRT((B33-$B$106)^2+(C33-$C$106)^2)</f>
+        <f t="shared" si="1"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="F33">
-        <f>SQRT((B33-$B$107)^2+(C33-$C$107)^2)</f>
+        <f t="shared" si="2"/>
         <v>20.248456731316587</v>
       </c>
       <c r="G33" t="str">
-        <f>IF(D33=MIN(D33:F33),"C1",IF(E33=MIN(D33:F33),"C2","C3"))</f>
+        <f t="shared" si="3"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1402,23 +1343,23 @@
         <v>73</v>
       </c>
       <c r="D34">
-        <f>SQRT((B34-$B$105)^2+(C34-$C$105)^2)</f>
+        <f t="shared" ref="D34:D65" si="4">SQRT((B34-$B$105)^2+(C34-$C$105)^2)</f>
         <v>29.120439557122072</v>
       </c>
       <c r="E34">
-        <f>SQRT((B34-$B$106)^2+(C34-$C$106)^2)</f>
+        <f t="shared" ref="E34:E65" si="5">SQRT((B34-$B$106)^2+(C34-$C$106)^2)</f>
         <v>8.5440037453175304</v>
       </c>
       <c r="F34">
-        <f>SQRT((B34-$B$107)^2+(C34-$C$107)^2)</f>
+        <f t="shared" ref="F34:F65" si="6">SQRT((B34-$B$107)^2+(C34-$C$107)^2)</f>
         <v>12.369316876852981</v>
       </c>
       <c r="G34" t="str">
-        <f>IF(D34=MIN(D34:F34),"C1",IF(E34=MIN(D34:F34),"C2","C3"))</f>
+        <f t="shared" ref="G34:G65" si="7">IF(D34=MIN(D34:F34),"C1",IF(E34=MIN(D34:F34),"C2","C3"))</f>
         <v>C2</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1429,23 +1370,23 @@
         <v>68</v>
       </c>
       <c r="D35">
-        <f>SQRT((B35-$B$105)^2+(C35-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>24.041630560342615</v>
       </c>
       <c r="E35">
-        <f>SQRT((B35-$B$106)^2+(C35-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>3.6055512754639891</v>
       </c>
       <c r="F35">
-        <f>SQRT((B35-$B$107)^2+(C35-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>17.464249196572979</v>
       </c>
       <c r="G35" t="str">
-        <f>IF(D35=MIN(D35:F35),"C1",IF(E35=MIN(D35:F35),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1456,23 +1397,23 @@
         <v>63</v>
       </c>
       <c r="D36">
-        <f>SQRT((B36-$B$105)^2+(C36-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>18.681541692269406</v>
       </c>
       <c r="E36">
-        <f>SQRT((B36-$B$106)^2+(C36-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="F36">
-        <f>SQRT((B36-$B$107)^2+(C36-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>22.803508501982758</v>
       </c>
       <c r="G36" t="str">
-        <f>IF(D36=MIN(D36:F36),"C1",IF(E36=MIN(D36:F36),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1483,23 +1424,23 @@
         <v>70</v>
       </c>
       <c r="D37">
-        <f>SQRT((B37-$B$105)^2+(C37-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>25.709920264364882</v>
       </c>
       <c r="E37">
-        <f>SQRT((B37-$B$106)^2+(C37-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>5.0990195135927845</v>
       </c>
       <c r="F37">
-        <f>SQRT((B37-$B$107)^2+(C37-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>15.811388300841896</v>
       </c>
       <c r="G37" t="str">
-        <f>IF(D37=MIN(D37:F37),"C1",IF(E37=MIN(D37:F37),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1510,23 +1451,23 @@
         <v>76</v>
       </c>
       <c r="D38">
-        <f>SQRT((B38-$B$105)^2+(C38-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>32.015621187164243</v>
       </c>
       <c r="E38">
-        <f>SQRT((B38-$B$106)^2+(C38-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>11.401754250991379</v>
       </c>
       <c r="F38">
-        <f>SQRT((B38-$B$107)^2+(C38-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>9.4868329805051381</v>
       </c>
       <c r="G38" t="str">
-        <f>IF(D38=MIN(D38:F38),"C1",IF(E38=MIN(D38:F38),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1537,23 +1478,23 @@
         <v>65</v>
       </c>
       <c r="D39">
-        <f>SQRT((B39-$B$105)^2+(C39-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>20.396078054371138</v>
       </c>
       <c r="E39">
-        <f>SQRT((B39-$B$106)^2+(C39-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="F39">
-        <f>SQRT((B39-$B$107)^2+(C39-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>21.189620100417091</v>
       </c>
       <c r="G39" t="str">
-        <f>IF(D39=MIN(D39:F39),"C1",IF(E39=MIN(D39:F39),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1564,23 +1505,23 @@
         <v>72</v>
       </c>
       <c r="D40">
-        <f>SQRT((B40-$B$105)^2+(C40-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>27.892651361962706</v>
       </c>
       <c r="E40">
-        <f>SQRT((B40-$B$106)^2+(C40-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>7.2801098892805181</v>
       </c>
       <c r="F40">
-        <f>SQRT((B40-$B$107)^2+(C40-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>13.601470508735444</v>
       </c>
       <c r="G40" t="str">
-        <f>IF(D40=MIN(D40:F40),"C1",IF(E40=MIN(D40:F40),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1591,23 +1532,23 @@
         <v>66</v>
       </c>
       <c r="D41">
-        <f>SQRT((B41-$B$105)^2+(C41-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>21.587033144922902</v>
       </c>
       <c r="E41">
-        <f>SQRT((B41-$B$106)^2+(C41-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="F41">
-        <f>SQRT((B41-$B$107)^2+(C41-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>19.924858845171276</v>
       </c>
       <c r="G41" t="str">
-        <f>IF(D41=MIN(D41:F41),"C1",IF(E41=MIN(D41:F41),"C2","C3"))</f>
+        <f t="shared" si="7"/>
         <v>C2</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1618,23 +1559,23 @@
         <v>78</v>
       </c>
       <c r="D42">
-        <f>SQRT((B42-$B$105)^2+(C42-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>34.205262752974143</v>
       </c>
       <c r="E42">
-        <f>SQRT((B42-$B$106)^2+(C42-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>13.601470508735444</v>
       </c>
       <c r="F42">
-        <f>SQRT((B42-$B$107)^2+(C42-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>7.2801098892805181</v>
       </c>
       <c r="G42" t="str">
-        <f>IF(D42=MIN(D42:F42),"C1",IF(E42=MIN(D42:F42),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1645,23 +1586,23 @@
         <v>80</v>
       </c>
       <c r="D43">
-        <f>SQRT((B43-$B$105)^2+(C43-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>36.400549446402593</v>
       </c>
       <c r="E43">
-        <f>SQRT((B43-$B$106)^2+(C43-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>15.811388300841896</v>
       </c>
       <c r="F43">
-        <f>SQRT((B43-$B$107)^2+(C43-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>5.0990195135927845</v>
       </c>
       <c r="G43" t="str">
-        <f>IF(D43=MIN(D43:F43),"C1",IF(E43=MIN(D43:F43),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1672,23 +1613,23 @@
         <v>85</v>
       </c>
       <c r="D44">
-        <f>SQRT((B44-$B$105)^2+(C44-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>41.484937025383083</v>
       </c>
       <c r="E44">
-        <f>SQRT((B44-$B$106)^2+(C44-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>20.880613017821101</v>
       </c>
       <c r="F44">
-        <f>SQRT((B44-$B$107)^2+(C44-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G44" t="str">
-        <f>IF(D44=MIN(D44:F44),"C1",IF(E44=MIN(D44:F44),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1699,23 +1640,23 @@
         <v>81</v>
       </c>
       <c r="D45">
-        <f>SQRT((B45-$B$105)^2+(C45-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>37.107950630558946</v>
       </c>
       <c r="E45">
-        <f>SQRT((B45-$B$106)^2+(C45-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>16.492422502470642</v>
       </c>
       <c r="F45">
-        <f>SQRT((B45-$B$107)^2+(C45-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>4.4721359549995796</v>
       </c>
       <c r="G45" t="str">
-        <f>IF(D45=MIN(D45:F45),"C1",IF(E45=MIN(D45:F45),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1726,23 +1667,23 @@
         <v>88</v>
       </c>
       <c r="D46">
-        <f>SQRT((B46-$B$105)^2+(C46-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>44.643028571099428</v>
       </c>
       <c r="E46">
-        <f>SQRT((B46-$B$106)^2+(C46-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>24.041630560342615</v>
       </c>
       <c r="F46">
-        <f>SQRT((B46-$B$107)^2+(C46-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>3.1622776601683795</v>
       </c>
       <c r="G46" t="str">
-        <f>IF(D46=MIN(D46:F46),"C1",IF(E46=MIN(D46:F46),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1753,23 +1694,23 @@
         <v>83</v>
       </c>
       <c r="D47">
-        <f>SQRT((B47-$B$105)^2+(C47-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>39.293765408776999</v>
       </c>
       <c r="E47">
-        <f>SQRT((B47-$B$106)^2+(C47-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>18.681541692269406</v>
       </c>
       <c r="F47">
-        <f>SQRT((B47-$B$107)^2+(C47-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>2.2360679774997898</v>
       </c>
       <c r="G47" t="str">
-        <f>IF(D47=MIN(D47:F47),"C1",IF(E47=MIN(D47:F47),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1780,23 +1721,23 @@
         <v>87</v>
       </c>
       <c r="D48">
-        <f>SQRT((B48-$B$105)^2+(C48-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>43.416586692184822</v>
       </c>
       <c r="E48">
-        <f>SQRT((B48-$B$106)^2+(C48-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>22.803508501982758</v>
       </c>
       <c r="F48">
-        <f>SQRT((B48-$B$107)^2+(C48-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="G48" t="str">
-        <f>IF(D48=MIN(D48:F48),"C1",IF(E48=MIN(D48:F48),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1807,23 +1748,23 @@
         <v>90</v>
       </c>
       <c r="D49">
-        <f>SQRT((B49-$B$105)^2+(C49-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>46.840153714521477</v>
       </c>
       <c r="E49">
-        <f>SQRT((B49-$B$106)^2+(C49-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>26.248809496813376</v>
       </c>
       <c r="F49">
-        <f>SQRT((B49-$B$107)^2+(C49-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>5.3851648071345037</v>
       </c>
       <c r="G49" t="str">
-        <f>IF(D49=MIN(D49:F49),"C1",IF(E49=MIN(D49:F49),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1834,23 +1775,23 @@
         <v>79</v>
       </c>
       <c r="D50">
-        <f>SQRT((B50-$B$105)^2+(C50-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>35.171010790137949</v>
       </c>
       <c r="E50">
-        <f>SQRT((B50-$B$106)^2+(C50-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>14.560219778561036</v>
       </c>
       <c r="F50">
-        <f>SQRT((B50-$B$107)^2+(C50-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>6.324555320336759</v>
       </c>
       <c r="G50" t="str">
-        <f>IF(D50=MIN(D50:F50),"C1",IF(E50=MIN(D50:F50),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1861,23 +1802,23 @@
         <v>86</v>
       </c>
       <c r="D51">
-        <f>SQRT((B51-$B$105)^2+(C51-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>42.720018726587654</v>
       </c>
       <c r="E51">
-        <f>SQRT((B51-$B$106)^2+(C51-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>22.135943621178654</v>
       </c>
       <c r="F51">
-        <f>SQRT((B51-$B$107)^2+(C51-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="G51" t="str">
-        <f>IF(D51=MIN(D51:F51),"C1",IF(E51=MIN(D51:F51),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1888,23 +1829,23 @@
         <v>84</v>
       </c>
       <c r="D52">
-        <f>SQRT((B52-$B$105)^2+(C52-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>40.26164427839479</v>
       </c>
       <c r="E52">
-        <f>SQRT((B52-$B$106)^2+(C52-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>19.646882704388499</v>
       </c>
       <c r="F52">
-        <f>SQRT((B52-$B$107)^2+(C52-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="G52" t="str">
-        <f>IF(D52=MIN(D52:F52),"C1",IF(E52=MIN(D52:F52),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1915,23 +1856,23 @@
         <v>82</v>
       </c>
       <c r="D53">
-        <f>SQRT((B53-$B$105)^2+(C53-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>38.600518131237564</v>
       </c>
       <c r="E53">
-        <f>SQRT((B53-$B$106)^2+(C53-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>18.027756377319946</v>
       </c>
       <c r="F53">
-        <f>SQRT((B53-$B$107)^2+(C53-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="G53" t="str">
-        <f>IF(D53=MIN(D53:F53),"C1",IF(E53=MIN(D53:F53),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1942,23 +1883,23 @@
         <v>92</v>
       </c>
       <c r="D54">
-        <f>SQRT((B54-$B$105)^2+(C54-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>49.040799340956916</v>
       </c>
       <c r="E54">
-        <f>SQRT((B54-$B$106)^2+(C54-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>28.460498941515414</v>
       </c>
       <c r="F54">
-        <f>SQRT((B54-$B$107)^2+(C54-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>7.6157731058639087</v>
       </c>
       <c r="G54" t="str">
-        <f>IF(D54=MIN(D54:F54),"C1",IF(E54=MIN(D54:F54),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1969,23 +1910,23 @@
         <v>89</v>
       </c>
       <c r="D55">
-        <f>SQRT((B55-$B$105)^2+(C55-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>45.880278987817846</v>
       </c>
       <c r="E55">
-        <f>SQRT((B55-$B$106)^2+(C55-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>25.298221281347036</v>
       </c>
       <c r="F55">
-        <f>SQRT((B55-$B$107)^2+(C55-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>4.4721359549995796</v>
       </c>
       <c r="G55" t="str">
-        <f>IF(D55=MIN(D55:F55),"C1",IF(E55=MIN(D55:F55),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1996,23 +1937,23 @@
         <v>80</v>
       </c>
       <c r="D56">
-        <f>SQRT((B56-$B$105)^2+(C56-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>36.138621999185304</v>
       </c>
       <c r="E56">
-        <f>SQRT((B56-$B$106)^2+(C56-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>15.524174696260024</v>
       </c>
       <c r="F56">
-        <f>SQRT((B56-$B$107)^2+(C56-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>5.3851648071345037</v>
       </c>
       <c r="G56" t="str">
-        <f>IF(D56=MIN(D56:F56),"C1",IF(E56=MIN(D56:F56),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2023,23 +1964,23 @@
         <v>91</v>
       </c>
       <c r="D57">
-        <f>SQRT((B57-$B$105)^2+(C57-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>47.539457296018853</v>
       </c>
       <c r="E57">
-        <f>SQRT((B57-$B$106)^2+(C57-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>26.92582403567252</v>
       </c>
       <c r="F57">
-        <f>SQRT((B57-$B$107)^2+(C57-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>6.0827625302982193</v>
       </c>
       <c r="G57" t="str">
-        <f>IF(D57=MIN(D57:F57),"C1",IF(E57=MIN(D57:F57),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2050,23 +1991,23 @@
         <v>86</v>
       </c>
       <c r="D58">
-        <f>SQRT((B58-$B$105)^2+(C58-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>42.201895692018383</v>
       </c>
       <c r="E58">
-        <f>SQRT((B58-$B$106)^2+(C58-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>21.587033144922902</v>
       </c>
       <c r="F58">
-        <f>SQRT((B58-$B$107)^2+(C58-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>1.4142135623730951</v>
       </c>
       <c r="G58" t="str">
-        <f>IF(D58=MIN(D58:F58),"C1",IF(E58=MIN(D58:F58),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2077,23 +2018,23 @@
         <v>88</v>
       </c>
       <c r="D59">
-        <f>SQRT((B59-$B$105)^2+(C59-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>44.384682042344295</v>
       </c>
       <c r="E59">
-        <f>SQRT((B59-$B$106)^2+(C59-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>23.769728648009426</v>
       </c>
       <c r="F59">
-        <f>SQRT((B59-$B$107)^2+(C59-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="G59" t="str">
-        <f>IF(D59=MIN(D59:F59),"C1",IF(E59=MIN(D59:F59),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2104,23 +2045,23 @@
         <v>94</v>
       </c>
       <c r="D60">
-        <f>SQRT((B60-$B$105)^2+(C60-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>51.244511901275828</v>
       </c>
       <c r="E60">
-        <f>SQRT((B60-$B$106)^2+(C60-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>30.675723300355934</v>
       </c>
       <c r="F60">
-        <f>SQRT((B60-$B$107)^2+(C60-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>9.8488578017961039</v>
       </c>
       <c r="G60" t="str">
-        <f>IF(D60=MIN(D60:F60),"C1",IF(E60=MIN(D60:F60),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2131,23 +2072,23 @@
         <v>91</v>
       </c>
       <c r="D61">
-        <f>SQRT((B61-$B$105)^2+(C61-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>47.801673610868477</v>
       </c>
       <c r="E61">
-        <f>SQRT((B61-$B$106)^2+(C61-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>27.202941017470888</v>
       </c>
       <c r="F61">
-        <f>SQRT((B61-$B$107)^2+(C61-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>6.324555320336759</v>
       </c>
       <c r="G61" t="str">
-        <f>IF(D61=MIN(D61:F61),"C1",IF(E61=MIN(D61:F61),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2158,23 +2099,23 @@
         <v>77</v>
       </c>
       <c r="D62">
-        <f>SQRT((B62-$B$105)^2+(C62-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>33.241540277189323</v>
       </c>
       <c r="E62">
-        <f>SQRT((B62-$B$106)^2+(C62-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>12.649110640673518</v>
       </c>
       <c r="F62">
-        <f>SQRT((B62-$B$107)^2+(C62-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>8.2462112512353212</v>
       </c>
       <c r="G62" t="str">
-        <f>IF(D62=MIN(D62:F62),"C1",IF(E62=MIN(D62:F62),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2185,23 +2126,23 @@
         <v>81</v>
       </c>
       <c r="D63">
-        <f>SQRT((B63-$B$105)^2+(C63-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>37.363083384538811</v>
       </c>
       <c r="E63">
-        <f>SQRT((B63-$B$106)^2+(C63-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>16.763054614240211</v>
       </c>
       <c r="F63">
-        <f>SQRT((B63-$B$107)^2+(C63-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>4.1231056256176606</v>
       </c>
       <c r="G63" t="str">
-        <f>IF(D63=MIN(D63:F63),"C1",IF(E63=MIN(D63:F63),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2212,23 +2153,23 @@
         <v>89</v>
       </c>
       <c r="D64">
-        <f>SQRT((B64-$B$105)^2+(C64-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>45.607017003965517</v>
       </c>
       <c r="E64">
-        <f>SQRT((B64-$B$106)^2+(C64-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>25</v>
       </c>
       <c r="F64">
-        <f>SQRT((B64-$B$107)^2+(C64-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>4.1231056256176606</v>
       </c>
       <c r="G64" t="str">
-        <f>IF(D64=MIN(D64:F64),"C1",IF(E64=MIN(D64:F64),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2239,23 +2180,23 @@
         <v>93</v>
       </c>
       <c r="D65">
-        <f>SQRT((B65-$B$105)^2+(C65-$C$105)^2)</f>
+        <f t="shared" si="4"/>
         <v>50</v>
       </c>
       <c r="E65">
-        <f>SQRT((B65-$B$106)^2+(C65-$C$106)^2)</f>
+        <f t="shared" si="5"/>
         <v>29.410882339705484</v>
       </c>
       <c r="F65">
-        <f>SQRT((B65-$B$107)^2+(C65-$C$107)^2)</f>
+        <f t="shared" si="6"/>
         <v>8.5440037453175304</v>
       </c>
       <c r="G65" t="str">
-        <f>IF(D65=MIN(D65:F65),"C1",IF(E65=MIN(D65:F65),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="7"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2266,23 +2207,23 @@
         <v>84</v>
       </c>
       <c r="D66">
-        <f>SQRT((B66-$B$105)^2+(C66-$C$105)^2)</f>
+        <f t="shared" ref="D66:D97" si="8">SQRT((B66-$B$105)^2+(C66-$C$105)^2)</f>
         <v>40.521599178709621</v>
       </c>
       <c r="E66">
-        <f>SQRT((B66-$B$106)^2+(C66-$C$106)^2)</f>
+        <f t="shared" ref="E66:E101" si="9">SQRT((B66-$B$106)^2+(C66-$C$106)^2)</f>
         <v>19.924858845171276</v>
       </c>
       <c r="F66">
-        <f>SQRT((B66-$B$107)^2+(C66-$C$107)^2)</f>
+        <f t="shared" ref="F66:F101" si="10">SQRT((B66-$B$107)^2+(C66-$C$107)^2)</f>
         <v>1</v>
       </c>
       <c r="G66" t="str">
-        <f>IF(D66=MIN(D66:F66),"C1",IF(E66=MIN(D66:F66),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G66:G97" si="11">IF(D66=MIN(D66:F66),"C1",IF(E66=MIN(D66:F66),"C2","C3"))</f>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2293,23 +2234,23 @@
         <v>88</v>
       </c>
       <c r="D67">
-        <f>SQRT((B67-$B$105)^2+(C67-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>44.922154890432402</v>
       </c>
       <c r="E67">
-        <f>SQRT((B67-$B$106)^2+(C67-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>24.351591323771842</v>
       </c>
       <c r="F67">
-        <f>SQRT((B67-$B$107)^2+(C67-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>3.6055512754639891</v>
       </c>
       <c r="G67" t="str">
-        <f>IF(D67=MIN(D67:F67),"C1",IF(E67=MIN(D67:F67),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2320,23 +2261,23 @@
         <v>95</v>
       </c>
       <c r="D68">
-        <f>SQRT((B68-$B$105)^2+(C68-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>52.201532544552748</v>
       </c>
       <c r="E68">
-        <f>SQRT((B68-$B$106)^2+(C68-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>31.622776601683793</v>
       </c>
       <c r="F68">
-        <f>SQRT((B68-$B$107)^2+(C68-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>10.770329614269007</v>
       </c>
       <c r="G68" t="str">
-        <f>IF(D68=MIN(D68:F68),"C1",IF(E68=MIN(D68:F68),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2347,23 +2288,23 @@
         <v>83</v>
       </c>
       <c r="D69">
-        <f>SQRT((B69-$B$105)^2+(C69-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>39.293765408776999</v>
       </c>
       <c r="E69">
-        <f>SQRT((B69-$B$106)^2+(C69-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>18.681541692269406</v>
       </c>
       <c r="F69">
-        <f>SQRT((B69-$B$107)^2+(C69-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>2.2360679774997898</v>
       </c>
       <c r="G69" t="str">
-        <f>IF(D69=MIN(D69:F69),"C1",IF(E69=MIN(D69:F69),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2374,23 +2315,23 @@
         <v>87</v>
       </c>
       <c r="D70">
-        <f>SQRT((B70-$B$105)^2+(C70-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>43.68065933568311</v>
       </c>
       <c r="E70">
-        <f>SQRT((B70-$B$106)^2+(C70-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>23.086792761230392</v>
       </c>
       <c r="F70">
-        <f>SQRT((B70-$B$107)^2+(C70-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>2.2360679774997898</v>
       </c>
       <c r="G70" t="str">
-        <f>IF(D70=MIN(D70:F70),"C1",IF(E70=MIN(D70:F70),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2401,23 +2342,23 @@
         <v>91</v>
       </c>
       <c r="D71">
-        <f>SQRT((B71-$B$105)^2+(C71-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>48.083261120685229</v>
       </c>
       <c r="E71">
-        <f>SQRT((B71-$B$106)^2+(C71-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>27.513632984395208</v>
       </c>
       <c r="F71">
-        <f>SQRT((B71-$B$107)^2+(C71-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>6.7082039324993694</v>
       </c>
       <c r="G71" t="str">
-        <f>IF(D71=MIN(D71:F71),"C1",IF(E71=MIN(D71:F71),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2428,23 +2369,23 @@
         <v>96</v>
       </c>
       <c r="D72">
-        <f>SQRT((B72-$B$105)^2+(C72-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>53.450912059571067</v>
       </c>
       <c r="E72">
-        <f>SQRT((B72-$B$106)^2+(C72-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>32.893768406797051</v>
       </c>
       <c r="F72">
-        <f>SQRT((B72-$B$107)^2+(C72-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>12.083045973594572</v>
       </c>
       <c r="G72" t="str">
-        <f>IF(D72=MIN(D72:F72),"C1",IF(E72=MIN(D72:F72),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2455,23 +2396,23 @@
         <v>93</v>
       </c>
       <c r="D73">
-        <f>SQRT((B73-$B$105)^2+(C73-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>50.289163842720633</v>
       </c>
       <c r="E73">
-        <f>SQRT((B73-$B$106)^2+(C73-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>29.732137494637012</v>
       </c>
       <c r="F73">
-        <f>SQRT((B73-$B$107)^2+(C73-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>8.9442719099991592</v>
       </c>
       <c r="G73" t="str">
-        <f>IF(D73=MIN(D73:F73),"C1",IF(E73=MIN(D73:F73),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2482,23 +2423,23 @@
         <v>97</v>
       </c>
       <c r="D74">
-        <f>SQRT((B74-$B$105)^2+(C74-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>54.708317466359723</v>
       </c>
       <c r="E74">
-        <f>SQRT((B74-$B$106)^2+(C74-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>34.176014981270121</v>
       </c>
       <c r="F74">
-        <f>SQRT((B74-$B$107)^2+(C74-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>13.416407864998739</v>
       </c>
       <c r="G74" t="str">
-        <f>IF(D74=MIN(D74:F74),"C1",IF(E74=MIN(D74:F74),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2509,23 +2450,23 @@
         <v>94</v>
       </c>
       <c r="D75">
-        <f>SQRT((B75-$B$105)^2+(C75-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>51.546095875439491</v>
       </c>
       <c r="E75">
-        <f>SQRT((B75-$B$106)^2+(C75-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>31.016124838541646</v>
       </c>
       <c r="F75">
-        <f>SQRT((B75-$B$107)^2+(C75-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>10.295630140987001</v>
       </c>
       <c r="G75" t="str">
-        <f>IF(D75=MIN(D75:F75),"C1",IF(E75=MIN(D75:F75),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2536,23 +2477,23 @@
         <v>90</v>
       </c>
       <c r="D76">
-        <f>SQRT((B76-$B$105)^2+(C76-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>47.127486671792717</v>
       </c>
       <c r="E76">
-        <f>SQRT((B76-$B$106)^2+(C76-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>26.570660511172846</v>
       </c>
       <c r="F76">
-        <f>SQRT((B76-$B$107)^2+(C76-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>5.8309518948453007</v>
       </c>
       <c r="G76" t="str">
-        <f>IF(D76=MIN(D76:F76),"C1",IF(E76=MIN(D76:F76),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2563,23 +2504,23 @@
         <v>96</v>
       </c>
       <c r="D77">
-        <f>SQRT((B77-$B$105)^2+(C77-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>53.160135440008048</v>
       </c>
       <c r="E77">
-        <f>SQRT((B77-$B$106)^2+(C77-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>32.572994949804659</v>
       </c>
       <c r="F77">
-        <f>SQRT((B77-$B$107)^2+(C77-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>11.704699910719626</v>
       </c>
       <c r="G77" t="str">
-        <f>IF(D77=MIN(D77:F77),"C1",IF(E77=MIN(D77:F77),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2590,23 +2531,23 @@
         <v>98</v>
       </c>
       <c r="D78">
-        <f>SQRT((B78-$B$105)^2+(C78-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>55.659680200302986</v>
       </c>
       <c r="E78">
-        <f>SQRT((B78-$B$106)^2+(C78-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>35.114099732158877</v>
       </c>
       <c r="F78">
-        <f>SQRT((B78-$B$107)^2+(C78-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>14.317821063276353</v>
       </c>
       <c r="G78" t="str">
-        <f>IF(D78=MIN(D78:F78),"C1",IF(E78=MIN(D78:F78),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2617,23 +2558,23 @@
         <v>95</v>
       </c>
       <c r="D79">
-        <f>SQRT((B79-$B$105)^2+(C79-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>52.497618993626752</v>
       </c>
       <c r="E79">
-        <f>SQRT((B79-$B$106)^2+(C79-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>31.953090617340916</v>
       </c>
       <c r="F79">
-        <f>SQRT((B79-$B$107)^2+(C79-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>11.180339887498949</v>
       </c>
       <c r="G79" t="str">
-        <f>IF(D79=MIN(D79:F79),"C1",IF(E79=MIN(D79:F79),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2644,23 +2585,23 @@
         <v>92</v>
       </c>
       <c r="D80">
-        <f>SQRT((B80-$B$105)^2+(C80-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>48.764741360946438</v>
       </c>
       <c r="E80">
-        <f>SQRT((B80-$B$106)^2+(C80-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>28.160255680657446</v>
       </c>
       <c r="F80">
-        <f>SQRT((B80-$B$107)^2+(C80-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>7.2801098892805181</v>
       </c>
       <c r="G80" t="str">
-        <f>IF(D80=MIN(D80:F80),"C1",IF(E80=MIN(D80:F80),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2671,23 +2612,23 @@
         <v>94</v>
       </c>
       <c r="D81">
-        <f>SQRT((B81-$B$105)^2+(C81-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>50.960769224963627</v>
       </c>
       <c r="E81">
-        <f>SQRT((B81-$B$106)^2+(C81-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>30.364452901377952</v>
       </c>
       <c r="F81">
-        <f>SQRT((B81-$B$107)^2+(C81-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>9.4868329805051381</v>
       </c>
       <c r="G81" t="str">
-        <f>IF(D81=MIN(D81:F81),"C1",IF(E81=MIN(D81:F81),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2698,23 +2639,23 @@
         <v>98</v>
       </c>
       <c r="D82">
-        <f>SQRT((B82-$B$105)^2+(C82-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>55.97320787662612</v>
       </c>
       <c r="E82">
-        <f>SQRT((B82-$B$106)^2+(C82-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>35.468295701936398</v>
       </c>
       <c r="F82">
-        <f>SQRT((B82-$B$107)^2+(C82-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>14.7648230602334</v>
       </c>
       <c r="G82" t="str">
-        <f>IF(D82=MIN(D82:F82),"C1",IF(E82=MIN(D82:F82),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2725,23 +2666,23 @@
         <v>96</v>
       </c>
       <c r="D83">
-        <f>SQRT((B83-$B$105)^2+(C83-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>53.758720222862451</v>
       </c>
       <c r="E83">
-        <f>SQRT((B83-$B$106)^2+(C83-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>33.241540277189323</v>
       </c>
       <c r="F83">
-        <f>SQRT((B83-$B$107)^2+(C83-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>12.529964086141668</v>
       </c>
       <c r="G83" t="str">
-        <f>IF(D83=MIN(D83:F83),"C1",IF(E83=MIN(D83:F83),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2752,23 +2693,23 @@
         <v>99</v>
       </c>
       <c r="D84">
-        <f>SQRT((B84-$B$105)^2+(C84-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>57.245087125446844</v>
       </c>
       <c r="E84">
-        <f>SQRT((B84-$B$106)^2+(C84-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>36.76955262170047</v>
       </c>
       <c r="F84">
-        <f>SQRT((B84-$B$107)^2+(C84-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>16.124515496597098</v>
       </c>
       <c r="G84" t="str">
-        <f>IF(D84=MIN(D84:F84),"C1",IF(E84=MIN(D84:F84),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2779,23 +2720,23 @@
         <v>97</v>
       </c>
       <c r="D85">
-        <f>SQRT((B85-$B$105)^2+(C85-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>55.027265968790417</v>
       </c>
       <c r="E85">
-        <f>SQRT((B85-$B$106)^2+(C85-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>34.539832078341085</v>
       </c>
       <c r="F85">
-        <f>SQRT((B85-$B$107)^2+(C85-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>13.892443989449804</v>
       </c>
       <c r="G85" t="str">
-        <f>IF(D85=MIN(D85:F85),"C1",IF(E85=MIN(D85:F85),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2806,23 +2747,23 @@
         <v>93</v>
       </c>
       <c r="D86">
-        <f>SQRT((B86-$B$105)^2+(C86-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>50.596442562694072</v>
       </c>
       <c r="E86">
-        <f>SQRT((B86-$B$106)^2+(C86-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>30.083217912982647</v>
       </c>
       <c r="F86">
-        <f>SQRT((B86-$B$107)^2+(C86-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>9.4339811320566032</v>
       </c>
       <c r="G86" t="str">
-        <f>IF(D86=MIN(D86:F86),"C1",IF(E86=MIN(D86:F86),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2833,23 +2774,23 @@
         <v>98</v>
       </c>
       <c r="D87">
-        <f>SQRT((B87-$B$105)^2+(C87-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>56.302753041036986</v>
       </c>
       <c r="E87">
-        <f>SQRT((B87-$B$106)^2+(C87-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>35.846896657869841</v>
       </c>
       <c r="F87">
-        <f>SQRT((B87-$B$107)^2+(C87-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>15.264337522473747</v>
       </c>
       <c r="G87" t="str">
-        <f>IF(D87=MIN(D87:F87),"C1",IF(E87=MIN(D87:F87),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2860,23 +2801,23 @@
         <v>95</v>
       </c>
       <c r="D88">
-        <f>SQRT((B88-$B$105)^2+(C88-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>52.810983706043572</v>
       </c>
       <c r="E88">
-        <f>SQRT((B88-$B$106)^2+(C88-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>32.310988842807021</v>
       </c>
       <c r="F88">
-        <f>SQRT((B88-$B$107)^2+(C88-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>11.661903789690601</v>
       </c>
       <c r="G88" t="str">
-        <f>IF(D88=MIN(D88:F88),"C1",IF(E88=MIN(D88:F88),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2887,23 +2828,23 @@
         <v>99</v>
       </c>
       <c r="D89">
-        <f>SQRT((B89-$B$105)^2+(C89-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>56.920997883030829</v>
       </c>
       <c r="E89">
-        <f>SQRT((B89-$B$106)^2+(C89-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>36.400549446402593</v>
       </c>
       <c r="F89">
-        <f>SQRT((B89-$B$107)^2+(C89-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>15.652475842498529</v>
       </c>
       <c r="G89" t="str">
-        <f>IF(D89=MIN(D89:F89),"C1",IF(E89=MIN(D89:F89),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2914,23 +2855,23 @@
         <v>100</v>
       </c>
       <c r="D90">
-        <f>SQRT((B90-$B$105)^2+(C90-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>58.523499553598128</v>
       </c>
       <c r="E90">
-        <f>SQRT((B90-$B$106)^2+(C90-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>38.078865529319543</v>
       </c>
       <c r="F90">
-        <f>SQRT((B90-$B$107)^2+(C90-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>17.4928556845359</v>
       </c>
       <c r="G90" t="str">
-        <f>IF(D90=MIN(D90:F90),"C1",IF(E90=MIN(D90:F90),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2941,23 +2882,23 @@
         <v>97</v>
       </c>
       <c r="D91">
-        <f>SQRT((B91-$B$105)^2+(C91-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>55.362442142665635</v>
       </c>
       <c r="E91">
-        <f>SQRT((B91-$B$106)^2+(C91-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>34.928498393145958</v>
       </c>
       <c r="F91">
-        <f>SQRT((B91-$B$107)^2+(C91-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>14.422205101855956</v>
       </c>
       <c r="G91" t="str">
-        <f>IF(D91=MIN(D91:F91),"C1",IF(E91=MIN(D91:F91),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2968,23 +2909,23 @@
         <v>92</v>
       </c>
       <c r="D92">
-        <f>SQRT((B92-$B$105)^2+(C92-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>49.33558553417604</v>
       </c>
       <c r="E92">
-        <f>SQRT((B92-$B$106)^2+(C92-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>28.792360097775937</v>
       </c>
       <c r="F92">
-        <f>SQRT((B92-$B$107)^2+(C92-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>8.0622577482985491</v>
       </c>
       <c r="G92" t="str">
-        <f>IF(D92=MIN(D92:F92),"C1",IF(E92=MIN(D92:F92),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2995,23 +2936,23 @@
         <v>98</v>
       </c>
       <c r="D93">
-        <f>SQRT((B93-$B$105)^2+(C93-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>55.659680200302986</v>
       </c>
       <c r="E93">
-        <f>SQRT((B93-$B$106)^2+(C93-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>35.114099732158877</v>
       </c>
       <c r="F93">
-        <f>SQRT((B93-$B$107)^2+(C93-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>14.317821063276353</v>
       </c>
       <c r="G93" t="str">
-        <f>IF(D93=MIN(D93:F93),"C1",IF(E93=MIN(D93:F93),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3022,23 +2963,23 @@
         <v>96</v>
       </c>
       <c r="D94">
-        <f>SQRT((B94-$B$105)^2+(C94-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>54.083269131959838</v>
       </c>
       <c r="E94">
-        <f>SQRT((B94-$B$106)^2+(C94-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>33.61547262794322</v>
       </c>
       <c r="F94">
-        <f>SQRT((B94-$B$107)^2+(C94-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>13.038404810405298</v>
       </c>
       <c r="G94" t="str">
-        <f>IF(D94=MIN(D94:F94),"C1",IF(E94=MIN(D94:F94),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3049,23 +2990,23 @@
         <v>99</v>
       </c>
       <c r="D95">
-        <f>SQRT((B95-$B$105)^2+(C95-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>57.584720195551874</v>
       </c>
       <c r="E95">
-        <f>SQRT((B95-$B$106)^2+(C95-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>37.161808352124091</v>
       </c>
       <c r="F95">
-        <f>SQRT((B95-$B$107)^2+(C95-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>16.643316977093239</v>
       </c>
       <c r="G95" t="str">
-        <f>IF(D95=MIN(D95:F95),"C1",IF(E95=MIN(D95:F95),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3076,23 +3017,23 @@
         <v>95</v>
       </c>
       <c r="D96">
-        <f>SQRT((B96-$B$105)^2+(C96-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>52.497618993626752</v>
       </c>
       <c r="E96">
-        <f>SQRT((B96-$B$106)^2+(C96-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>31.953090617340916</v>
       </c>
       <c r="F96">
-        <f>SQRT((B96-$B$107)^2+(C96-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>11.180339887498949</v>
       </c>
       <c r="G96" t="str">
-        <f>IF(D96=MIN(D96:F96),"C1",IF(E96=MIN(D96:F96),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3103,23 +3044,23 @@
         <v>100</v>
       </c>
       <c r="D97">
-        <f>SQRT((B97-$B$105)^2+(C97-$C$105)^2)</f>
+        <f t="shared" si="8"/>
         <v>58.189346103904619</v>
       </c>
       <c r="E97">
-        <f>SQRT((B97-$B$106)^2+(C97-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>37.696153649941529</v>
       </c>
       <c r="F97">
-        <f>SQRT((B97-$B$107)^2+(C97-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>17</v>
       </c>
       <c r="G97" t="str">
-        <f>IF(D97=MIN(D97:F97),"C1",IF(E97=MIN(D97:F97),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="11"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3130,23 +3071,23 @@
         <v>97</v>
       </c>
       <c r="D98">
-        <f>SQRT((B98-$B$105)^2+(C98-$C$105)^2)</f>
+        <f t="shared" ref="D98:D129" si="12">SQRT((B98-$B$105)^2+(C98-$C$105)^2)</f>
         <v>54.708317466359723</v>
       </c>
       <c r="E98">
-        <f>SQRT((B98-$B$106)^2+(C98-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>34.176014981270121</v>
       </c>
       <c r="F98">
-        <f>SQRT((B98-$B$107)^2+(C98-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>13.416407864998739</v>
       </c>
       <c r="G98" t="str">
-        <f>IF(D98=MIN(D98:F98),"C1",IF(E98=MIN(D98:F98),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" ref="G98:G129" si="13">IF(D98=MIN(D98:F98),"C1",IF(E98=MIN(D98:F98),"C2","C3"))</f>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3157,23 +3098,23 @@
         <v>98</v>
       </c>
       <c r="D99">
-        <f>SQRT((B99-$B$105)^2+(C99-$C$105)^2)</f>
+        <f t="shared" si="12"/>
         <v>55.97320787662612</v>
       </c>
       <c r="E99">
-        <f>SQRT((B99-$B$106)^2+(C99-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>35.468295701936398</v>
       </c>
       <c r="F99">
-        <f>SQRT((B99-$B$107)^2+(C99-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>14.7648230602334</v>
       </c>
       <c r="G99" t="str">
-        <f>IF(D99=MIN(D99:F99),"C1",IF(E99=MIN(D99:F99),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="13"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3184,23 +3125,23 @@
         <v>100</v>
       </c>
       <c r="D100">
-        <f>SQRT((B100-$B$105)^2+(C100-$C$105)^2)</f>
+        <f t="shared" si="12"/>
         <v>58.523499553598128</v>
       </c>
       <c r="E100">
-        <f>SQRT((B100-$B$106)^2+(C100-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>38.078865529319543</v>
       </c>
       <c r="F100">
-        <f>SQRT((B100-$B$107)^2+(C100-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>17.4928556845359</v>
       </c>
       <c r="G100" t="str">
-        <f>IF(D100=MIN(D100:F100),"C1",IF(E100=MIN(D100:F100),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="13"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3211,41 +3152,41 @@
         <v>99</v>
       </c>
       <c r="D101">
-        <f>SQRT((B101-$B$105)^2+(C101-$C$105)^2)</f>
+        <f t="shared" si="12"/>
         <v>57.9396237474839</v>
       </c>
       <c r="E101">
-        <f>SQRT((B101-$B$106)^2+(C101-$C$106)^2)</f>
+        <f t="shared" si="9"/>
         <v>37.576588456111871</v>
       </c>
       <c r="F101">
-        <f>SQRT((B101-$B$107)^2+(C101-$C$107)^2)</f>
+        <f t="shared" si="10"/>
         <v>17.204650534085253</v>
       </c>
       <c r="G101" t="str">
-        <f>IF(D101=MIN(D101:F101),"C1",IF(E101=MIN(D101:F101),"C2","C3"))</f>
-        <v>C3</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+        <f t="shared" si="13"/>
+        <v>C3</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B105">
         <v>3</v>
@@ -3254,9 +3195,9 @@
         <v>45</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B106">
         <v>8</v>
@@ -3265,9 +3206,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B107">
         <v>14</v>
@@ -3276,14 +3217,14 @@
         <v>85</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>14</v>
@@ -3292,9 +3233,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B111">
         <f>AVERAGEIF($G$2:$G$101,"C1",$B$2:$B$101)</f>
@@ -3305,9 +3246,9 @@
         <v>48.588235294117645</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B112">
         <f>AVERAGEIF($G$2:$G$101,"C2",$B$2:$B$101)</f>
@@ -3318,9 +3259,9 @@
         <v>66.36363636363636</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="B113">
         <f>AVERAGEIF($G$2:$G$101,"C3",$B$2:$B$101)</f>
@@ -3335,101 +3276,4 @@
   <autoFilter ref="A1:G101" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="23.9453125" customWidth="1"/>
-    <col min="2" max="2" width="99.94921875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="3"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>